<commit_message>
update mode validation (#301) a62df42df267f94ed02538c9220b50e4b7c7e572
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-fr-core-cs-mode-validation-identity.xlsx
+++ b/main/ig/CodeSystem-fr-core-cs-mode-validation-identity.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="72">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-28T14:22:24+00:00</t>
+    <t>2026-06-12T14:04:24+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -126,7 +126,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>13</t>
+    <t>14</t>
   </si>
   <si>
     <t>Level</t>
@@ -162,64 +162,73 @@
     <t>Carte Européenne</t>
   </si>
   <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>Carte nationale d'identité</t>
+  </si>
+  <si>
+    <t>LE</t>
+  </si>
+  <si>
+    <t>Livret de famille</t>
+  </si>
+  <si>
+    <t>PA</t>
+  </si>
+  <si>
+    <t>Passeport</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>Permis de conduire</t>
+  </si>
+  <si>
+    <t>TC</t>
+  </si>
+  <si>
+    <t>Tiers de confiance</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>Acte de naissance + Carte vitale avec photo</t>
+  </si>
+  <si>
+    <t>AV</t>
+  </si>
+  <si>
+    <t>Application Carte Vitale</t>
+  </si>
+  <si>
+    <t>CS</t>
+  </si>
+  <si>
+    <t>Carte de séjour</t>
+  </si>
+  <si>
+    <t>Carte de séjour ou titre de séjour</t>
+  </si>
+  <si>
+    <t>IE</t>
+  </si>
+  <si>
+    <t>Identification électronique EIDAS</t>
+  </si>
+  <si>
+    <t>DC</t>
+  </si>
+  <si>
+    <t>Document de Circulation pour étranger mineur</t>
+  </si>
+  <si>
     <t>CM</t>
   </si>
   <si>
     <t>Carte militaire</t>
-  </si>
-  <si>
-    <t>CN</t>
-  </si>
-  <si>
-    <t>Carte nationale d'identité</t>
-  </si>
-  <si>
-    <t>CS</t>
-  </si>
-  <si>
-    <t>Carte de séjour</t>
-  </si>
-  <si>
-    <t>LE</t>
-  </si>
-  <si>
-    <t>Livret de famille</t>
-  </si>
-  <si>
-    <t>PA</t>
-  </si>
-  <si>
-    <t>Passeport</t>
-  </si>
-  <si>
-    <t>PC</t>
-  </si>
-  <si>
-    <t>Permis de conduire</t>
-  </si>
-  <si>
-    <t>TC</t>
-  </si>
-  <si>
-    <t>Tiers de confiance</t>
-  </si>
-  <si>
-    <t>DC</t>
-  </si>
-  <si>
-    <t>Document de Circulation pour étranger mineur</t>
-  </si>
-  <si>
-    <t>AC</t>
-  </si>
-  <si>
-    <t>Acte de naissance + Carte vitale avec photo</t>
-  </si>
-  <si>
-    <t>IE</t>
-  </si>
-  <si>
-    <t>Identification électronique EIDAS</t>
   </si>
 </sst>
 </file>
@@ -537,7 +546,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -705,7 +714,7 @@
         <v>64</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13">
@@ -713,13 +722,13 @@
         <v>42</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14">
@@ -727,13 +736,27 @@
         <v>42</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>68</v>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="2">
+        <v>42</v>
+      </c>
+      <c r="B15" t="s" s="2">
+        <v>70</v>
+      </c>
+      <c r="C15" t="s" s="2">
+        <v>71</v>
+      </c>
+      <c r="D15" t="s" s="2">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>